<commit_message>
Rename and support any LED
</commit_message>
<xml_diff>
--- a/pinout/bom_arduino_nano.xlsx
+++ b/pinout/bom_arduino_nano.xlsx
@@ -8,17 +8,28 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\JD\Montmorency\git\MO_34A_Labs\pinout\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6430E65A-9B9F-49D4-B412-32250B0C26C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD2A8CBF-D58B-4454-8C6A-251E41E745E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2595" yWindow="1605" windowWidth="21600" windowHeight="12690" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -246,7 +257,7 @@
     <t>D3, RX,TX</t>
   </si>
   <si>
-    <t>LED Green 0805</t>
+    <t>LED Green/Yellow/Blue/Red 0805</t>
   </si>
 </sst>
 </file>
@@ -295,13 +306,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -588,424 +598,421 @@
   <dimension ref="A1:F22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="1" max="1" width="17.42578125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="45.85546875" customWidth="1"/>
     <col min="5" max="5" width="27.7109375" customWidth="1"/>
     <col min="6" max="6" width="36.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="2" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+      <c r="A2" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="1"/>
-      <c r="C2" s="1" t="s">
+      <c r="C2" t="s">
         <v>11</v>
       </c>
-      <c r="D2" s="2">
-        <v>1</v>
-      </c>
-      <c r="E2" s="1" t="s">
+      <c r="D2" s="1">
+        <v>1</v>
+      </c>
+      <c r="E2" t="s">
         <v>12</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="F2" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B3" s="2"/>
-      <c r="C3" s="2" t="s">
+      <c r="B3" s="1"/>
+      <c r="C3" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D3" s="2">
-        <v>1</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F3" s="4" t="s">
+      <c r="D3" s="1">
+        <v>1</v>
+      </c>
+      <c r="E3" t="s">
+        <v>6</v>
+      </c>
+      <c r="F3" s="3" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B4" s="2"/>
-      <c r="C4" s="2" t="s">
+      <c r="B4" s="1"/>
+      <c r="C4" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="D4" s="2">
-        <v>1</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F4" s="4" t="s">
+      <c r="D4" s="1">
+        <v>1</v>
+      </c>
+      <c r="E4" t="s">
+        <v>6</v>
+      </c>
+      <c r="F4" s="3" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B5" s="2"/>
-      <c r="C5" s="2" t="s">
+      <c r="B5" s="1"/>
+      <c r="C5" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="D5" s="2">
-        <v>6</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F5" s="4" t="s">
+      <c r="D5" s="1">
+        <v>6</v>
+      </c>
+      <c r="E5" t="s">
+        <v>6</v>
+      </c>
+      <c r="F5" s="3" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A6" s="2" t="s">
+      <c r="A6" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B6" s="2"/>
-      <c r="C6" s="2" t="s">
+      <c r="B6" s="1"/>
+      <c r="C6" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="D6" s="2">
+      <c r="D6" s="1">
         <v>3</v>
       </c>
-      <c r="E6" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F6" s="4" t="s">
+      <c r="E6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F6" s="3" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A7" s="2" t="s">
+      <c r="A7" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B7" s="2"/>
-      <c r="C7" s="2" t="s">
+      <c r="B7" s="1"/>
+      <c r="C7" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="D7" s="2">
-        <v>1</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F7" s="4" t="s">
+      <c r="D7" s="1">
+        <v>1</v>
+      </c>
+      <c r="E7" t="s">
+        <v>6</v>
+      </c>
+      <c r="F7" s="3" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A8" s="2" t="s">
+      <c r="A8" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="2"/>
-      <c r="C8" s="2" t="s">
+      <c r="B8" s="1"/>
+      <c r="C8" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="D8" s="2">
-        <v>1</v>
-      </c>
-      <c r="E8" s="4" t="s">
+      <c r="D8" s="1">
+        <v>1</v>
+      </c>
+      <c r="E8" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="F8" s="4" t="s">
+      <c r="F8" s="3" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A9" s="2" t="s">
+      <c r="A9" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="C9" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="D9" s="2">
-        <v>1</v>
-      </c>
-      <c r="E9" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F9" s="4" t="s">
+      <c r="D9" s="1">
+        <v>1</v>
+      </c>
+      <c r="E9" t="s">
+        <v>6</v>
+      </c>
+      <c r="F9" s="3" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A10" s="2" t="s">
+      <c r="A10" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="C10" s="2"/>
-      <c r="D10" s="2">
-        <v>1</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F10" s="4" t="s">
+      <c r="C10" s="1"/>
+      <c r="D10" s="1">
+        <v>1</v>
+      </c>
+      <c r="E10" t="s">
+        <v>6</v>
+      </c>
+      <c r="F10" s="3" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A11" s="2" t="s">
+      <c r="A11" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2">
-        <v>1</v>
-      </c>
-      <c r="E11" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F11" s="4" t="s">
+      <c r="C11" s="1"/>
+      <c r="D11" s="1">
+        <v>1</v>
+      </c>
+      <c r="E11" t="s">
+        <v>6</v>
+      </c>
+      <c r="F11" s="3" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A12" s="2" t="s">
+      <c r="A12" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="C12" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="D12" s="2">
+      <c r="D12" s="1">
         <v>4</v>
       </c>
-      <c r="E12" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="F12" s="4" t="s">
+      <c r="E12" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="F12" s="3" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A13" s="2" t="s">
+      <c r="A13" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B13" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="C13" s="2" t="s">
+      <c r="C13" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="D13" s="2">
+      <c r="D13" s="1">
         <v>4</v>
       </c>
-      <c r="E13" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="F13" s="4" t="s">
+      <c r="E13" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="F13" s="3" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A14" s="2" t="s">
+      <c r="A14" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B14" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="C14" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="D14" s="2">
-        <v>1</v>
-      </c>
-      <c r="E14" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="F14" s="4" t="s">
+      <c r="D14" s="1">
+        <v>1</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="F14" s="3" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A15" s="2" t="s">
+      <c r="A15" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="B15" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="C15" s="2" t="s">
+      <c r="C15" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="D15" s="2">
-        <v>1</v>
-      </c>
-      <c r="E15" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="F15" s="4" t="s">
+      <c r="D15" s="1">
+        <v>1</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="F15" s="3" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A16" s="2" t="s">
+      <c r="A16" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="B16" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="C16" s="2" t="s">
+      <c r="C16" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="D16" s="2">
+      <c r="D16" s="1">
         <v>2</v>
       </c>
-      <c r="E16" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="F16" s="4" t="s">
+      <c r="E16" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="F16" s="3" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A17" s="2" t="s">
+      <c r="A17" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="B17" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="C17" s="2" t="s">
+      <c r="C17" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="D17" s="2">
+      <c r="D17" s="1">
         <v>2</v>
       </c>
-      <c r="E17" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="F17" s="4" t="s">
+      <c r="E17" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="F17" s="3" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A18" s="2" t="s">
+      <c r="A18" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="B18" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="C18" s="2" t="s">
+      <c r="C18" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="D18" s="2">
-        <v>1</v>
-      </c>
-      <c r="E18" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="F18" s="4" t="s">
+      <c r="D18" s="1">
+        <v>1</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="F18" s="3" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="19" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A19" s="2" t="s">
+      <c r="A19" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="B19" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="C19" s="2" t="s">
+      <c r="C19" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="D19" s="2">
+      <c r="D19" s="1">
         <v>5</v>
       </c>
-      <c r="E19" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="F19" s="4" t="s">
+      <c r="E19" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="F19" s="3" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="20" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A20" s="3" t="s">
+      <c r="A20" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B20" s="1"/>
-      <c r="C20" s="3" t="s">
+      <c r="C20" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="D20" s="3">
-        <v>1</v>
-      </c>
-      <c r="E20" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="F20" s="4" t="s">
+      <c r="D20" s="2">
+        <v>1</v>
+      </c>
+      <c r="E20" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="F20" s="3" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="21" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A21" s="3" t="s">
+      <c r="A21" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="B21" s="1"/>
-      <c r="C21" s="3" t="s">
+      <c r="C21" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="D21" s="3">
+      <c r="D21" s="2">
         <v>2</v>
       </c>
-      <c r="E21" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="F21" s="4" t="s">
+      <c r="E21" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="F21" s="3" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="22" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A22" s="3" t="s">
+      <c r="A22" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="B22" s="1"/>
-      <c r="C22" s="3" t="s">
+      <c r="C22" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="D22" s="3">
+      <c r="D22" s="2">
         <v>3</v>
       </c>
-      <c r="E22" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="F22" s="1" t="s">
+      <c r="E22" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="F22" t="s">
         <v>7</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update datasheet and doc
</commit_message>
<xml_diff>
--- a/pinout/bom_arduino_nano.xlsx
+++ b/pinout/bom_arduino_nano.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\JD\Montmorency\git\MO_34A_Labs\pinout\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD2A8CBF-D58B-4454-8C6A-251E41E745E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AEDE2BA-0C2F-4DFB-81EE-C93CD896AE98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2595" yWindow="1605" windowWidth="21600" windowHeight="12690" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -116,12 +116,6 @@
     <t>U1</t>
   </si>
   <si>
-    <t>ATMega328PB-A</t>
-  </si>
-  <si>
-    <t>556-ATMEGA328PB-AU</t>
-  </si>
-  <si>
     <t>CH340G</t>
   </si>
   <si>
@@ -258,6 +252,12 @@
   </si>
   <si>
     <t>LED Green/Yellow/Blue/Red 0805</t>
+  </si>
+  <si>
+    <t>ATMega328P-A</t>
+  </si>
+  <si>
+    <t>556-ATMEGA328P-AU</t>
   </si>
 </sst>
 </file>
@@ -719,7 +719,7 @@
       </c>
       <c r="B7" s="1"/>
       <c r="C7" s="1" t="s">
-        <v>26</v>
+        <v>72</v>
       </c>
       <c r="D7" s="1">
         <v>1</v>
@@ -728,7 +728,7 @@
         <v>6</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>27</v>
+        <v>73</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
@@ -737,44 +737,44 @@
       </c>
       <c r="B8" s="1"/>
       <c r="C8" s="1" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="D8" s="1">
         <v>1</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C9" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="D9" s="1">
+        <v>1</v>
+      </c>
+      <c r="E9" t="s">
+        <v>6</v>
+      </c>
+      <c r="F9" s="3" t="s">
         <v>31</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="D9" s="1">
-        <v>1</v>
-      </c>
-      <c r="E9" t="s">
-        <v>6</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C10" s="1"/>
       <c r="D10" s="1">
@@ -784,15 +784,15 @@
         <v>6</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C11" s="1"/>
       <c r="D11" s="1">
@@ -802,18 +802,18 @@
         <v>6</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C12" s="1" t="s">
         <v>40</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>42</v>
       </c>
       <c r="D12" s="1">
         <v>4</v>
@@ -822,18 +822,18 @@
         <v>6</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C13" s="1" t="s">
         <v>44</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>46</v>
       </c>
       <c r="D13" s="1">
         <v>4</v>
@@ -842,58 +842,58 @@
         <v>6</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C14" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="D14" s="1">
+        <v>1</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="F14" s="3" t="s">
         <v>49</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="D14" s="1">
-        <v>1</v>
-      </c>
-      <c r="E14" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="F14" s="3" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D15" s="1">
+        <v>1</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="F15" s="3" t="s">
         <v>52</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="D15" s="1">
-        <v>1</v>
-      </c>
-      <c r="E15" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="F15" s="3" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="D16" s="1">
         <v>2</v>
@@ -902,18 +902,18 @@
         <v>6</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="D17" s="1">
         <v>2</v>
@@ -922,38 +922,38 @@
         <v>6</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D18" s="1">
+        <v>1</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="F18" s="3" t="s">
         <v>61</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="D18" s="1">
-        <v>1</v>
-      </c>
-      <c r="E18" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="F18" s="3" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="19" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="D19" s="1">
         <v>5</v>
@@ -962,7 +962,7 @@
         <v>6</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="20" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
@@ -970,7 +970,7 @@
         <v>8</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="D20" s="2">
         <v>1</v>
@@ -979,15 +979,15 @@
         <v>6</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="21" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="D21" s="2">
         <v>2</v>
@@ -996,15 +996,15 @@
         <v>6</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="22" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="D22" s="2">
         <v>3</v>

</xml_diff>